<commit_message>
US-01: Recibir PDF por API
POST /manuscripts multipart con token de servicio, validación de firma
%PDF- y tamaño (25 MB), modelo Manuscript con migración Alembic,
almacenamiento en storage/{id}.pdf, idempotencia por submission_id +
sha256 (D-01) y análisis lanzado con BackgroundTasks (D-04).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/priorizacion_rice_sprint1.xlsx
+++ b/priorizacion_rice_sprint1.xlsx
@@ -6471,7 +6471,7 @@
       </c>
       <c r="E13" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F13" s="61" t="n"/>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="E14" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F14" s="61" t="n"/>
@@ -6523,7 +6523,7 @@
       </c>
       <c r="E15" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F15" s="61" t="n"/>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="E16" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F16" s="61" t="n"/>

</xml_diff>

<commit_message>
US-04: Extraer texto y páginas
extract_text(pdf) con PyMuPDF: páginas, bloques con bbox, fuente, tamaño,
negrita y cursiva, texto plano por página; detección de PDF escaneado,
corrupto o cifrado → unreadable con motivo (ALT-01); modelo Document
JSON/JSONB con migración y etapa de extracción en el pipeline.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/priorizacion_rice_sprint1.xlsx
+++ b/priorizacion_rice_sprint1.xlsx
@@ -6575,7 +6575,7 @@
       </c>
       <c r="E17" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F17" s="61" t="n"/>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="E18" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F18" s="61" t="n"/>
@@ -6627,7 +6627,7 @@
       </c>
       <c r="E19" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F19" s="61" t="n"/>
@@ -6653,7 +6653,7 @@
       </c>
       <c r="E20" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F20" s="61" t="n"/>

</xml_diff>

<commit_message>
US-09: Cargar reglas Innosoft desde YAML
rules/innosoft/figuras.yaml con RE-20..RE-27, registro de evaluadores
con parámetros Pydantic, loader con JSON Schema y validaciones
adicionales (id único, categoría, evaluador, marcadores, parámetros),
rules_hash, carga al arrancar que detiene la API si hay reglas
inválidas y GET /rules?section=&categoria=.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/priorizacion_rice_sprint1.xlsx
+++ b/priorizacion_rice_sprint1.xlsx
@@ -6679,7 +6679,7 @@
       </c>
       <c r="E21" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F21" s="61" t="n"/>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="E22" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F22" s="61" t="n"/>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="E23" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F23" s="61" t="n"/>
@@ -6757,7 +6757,7 @@
       </c>
       <c r="E24" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F24" s="61" t="n"/>

</xml_diff>

<commit_message>
US-06: Extraer figuras: posición, tamaño y pie
extract_figures(pdf, document): imágenes raster por ocurrencia con bbox,
píxeles reales y DPI efectivo; dibujos vectoriales agrupados por región
(kind=vector, sin DPI); filtro de imágenes decorativas (< 1 % del área);
pie de figura debajo o arriba con tolerancia de 40 pt y regex tolerante;
fusión de mosaicos que comparten pie; miniaturas en storage/{id}/fig-n.png;
etapa de figuras en el pipeline.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/priorizacion_rice_sprint1.xlsx
+++ b/priorizacion_rice_sprint1.xlsx
@@ -6783,7 +6783,7 @@
       </c>
       <c r="E25" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F25" s="61" t="n"/>
@@ -6809,7 +6809,7 @@
       </c>
       <c r="E26" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F26" s="61" t="n"/>
@@ -6835,7 +6835,7 @@
       </c>
       <c r="E27" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F27" s="61" t="n"/>
@@ -6861,7 +6861,7 @@
       </c>
       <c r="E28" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F28" s="61" t="n"/>
@@ -6887,7 +6887,7 @@
       </c>
       <c r="E29" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F29" s="61" t="n"/>

</xml_diff>

<commit_message>
US-10: Validar figuras: tamaño y proporción
Motor run_rules(context, rules) con aislamiento por regla (rule_error),
evaluadores figure_min_pixels (RE-20) y figure_min_dpi (RE-21) con
umbrales solo en YAML, tabla findings con migración, etapa de validación
en el pipeline, GET /manuscripts/{id}/findings y pruebas por regla en
tests/rules/ con verificación de cobertura (formato-reglas §14).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/priorizacion_rice_sprint1.xlsx
+++ b/priorizacion_rice_sprint1.xlsx
@@ -6913,7 +6913,7 @@
       </c>
       <c r="E30" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F30" s="61" t="n"/>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E31" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F31" s="61" t="n"/>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="E32" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F32" s="61" t="n"/>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="E33" s="68" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F33" s="61" t="n"/>

</xml_diff>